<commit_message>
updated notebook, application, expanded data files
</commit_message>
<xml_diff>
--- a/data/skin.xlsx
+++ b/data/skin.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nayeliguzman/Documents/cosmetic-ingredient-analyzer/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{699E146D-5CB1-8A4A-9449-4453AC2D1579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD04487-EEF9-9046-ACE5-A46F2D3CA78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24680" yWindow="4620" windowWidth="36260" windowHeight="18080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="55">
   <si>
     <t>Product</t>
   </si>
@@ -173,13 +173,25 @@
   </si>
   <si>
     <t>CHANEL sublimage lessence de teint</t>
+  </si>
+  <si>
+    <t>LilyAna Vitamin C Serum</t>
+  </si>
+  <si>
+    <t>Aqua (Deionized Water), Aloe Barbadensis Leaf (Organic Aloe) Juice, Sodium Ascorbyl Phosphate (Vitamin C), Dimethyl Sulfone (MSM), Acrylates/C10-30 Alkyl Acrylate Crosspolymer, Tocopheryl Acetate (Vitamin E), Simmondsia Chinensis (Organic Jojoba) Seed Oil, Sodium Hydroxide, Glycerin (Kosher, Vegetable), Caesalpinia Spinosa Gum (Tara, Botanical Hyaluronic Acid), Potassium Sorbate, Sodium Benzoate, Alcohol, Equisetum Arvense (Horsetail) Extract, Taraxacum Officinale (Organic Dandelion) Extract, Centella Asiatica (Organic Gotu Kola) Extract, Geranium Maculatum (Wild Geranium) Extract, Phenoxyethanol, Ethylhexylglycerin</t>
+  </si>
+  <si>
+    <t>Medik8 Retinol</t>
+  </si>
+  <si>
+    <t>Aqua (Water), Caprylic/Capric Triglyceride, Glycerin, Isododecane, Cetearyl Olivate, Sodium Acrylate/Sodium Acryloyldimethyl Taurate Copolymer, Cetearyl Alcohol, PPG-12/SMDI Copolymer, Sorbitan Olivate, Tocopheryl Acetate, Titanium Dioxide, Eclipta Prostrata Extract, Cyclodextrin, Squalane, Hydroxyethyl Acrylate/Sodium Acryloyldimethyl Taurate Copolymer, Phenoxyethanol, Melia Azadirachta Leaf Extract, Hydroxypropyl Methylcellulose, Sodium Hyaluronate, Tetrahexyldecyl Ascorbate, Rubus Chamaemorus (Cloudberry) Seed Oil, Alumina, Isostearic Acid, Lecithin, Polyglyceryl-3 Polyricinoleate, Polyhydroxystearic Acid, Stearic Acid, Pentylene Glycol, Retinal, Moringa Oleifera Seed Oil, Sodium Polyaspartate, Climbazole, Disodium EDTA, Lonicera Japonica (Honeysuckle) Flower Extract, Lonicera Caprifolium (Honeysuckle) Flower Extract, Daucus Carota Sativa (Carrot) Seed Oil, Ethylhexylglycerin, 3-O-Ethyl Ascorbic Acid, Dipteryx Odorata (Tonka) Bean Extract, Hydroxyacetophenone, Polysorbate 60, Sorbitan Isostearate, Vanilla Planifolia (Vanilla) Fruit Extract, Decylene Glycol, 1,2-Hexanediol, BHT, Coumarin.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -239,6 +251,18 @@
       <name val="Helvetica Neue"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF262626"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -386,7 +410,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -452,6 +476,12 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1583,7 +1613,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T23"/>
+  <dimension ref="A1:T25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.33203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="42.5" style="1" customWidth="1"/>
@@ -2169,6 +2199,22 @@
         <v>49</v>
       </c>
     </row>
+    <row r="24" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="22" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" ht="20" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="23" t="s">
+        <v>54</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>

</xml_diff>